<commit_message>
feat: 6 business models + hardware specs — SaaS, Mac Mini, pay-per-use, hybrid, BYOK, consulting
</commit_message>
<xml_diff>
--- a/packages/dashboard-v2/public/paganini-cost-model.xlsx
+++ b/packages/dashboard-v2/public/paganini-cost-model.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Tech Stack Atual" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Retroativo (32 dias)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Custo de Vida CTO SP" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Cenários de Venda" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Modelos de Negócio" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Referências" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Hardware Specs" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +77,22 @@
       <color rgb="00DC2626"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0016A34A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0016A34A"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +123,12 @@
         <bgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+        <bgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -134,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -154,6 +175,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3599,593 +3624,1970 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Modelo de Negócio</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>POC (1 fundo)</t>
+          <t>Como funciona</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Produção (3-5 fundos)</t>
+          <t>CAPEX (upfront)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Enterprise (10+)</t>
+          <t>OPEX/mês</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Custo/task</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Break-even</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Risco nosso</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Risco cliente</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>📊 Parâmetros</t>
+          <t>🅰 SaaS CLOUD — Nós hospedamos, cliente assina</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Fundos ativos</t>
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Descrição</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>10+</t>
-        </is>
-      </c>
+          <t>EKS managed na AWS sa-east-1. Multi-tenant. Nós operamos tudo.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Usuários</t>
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Infra nosso</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>EKS cluster + RDS + ALB + NAT + monitoring</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>50+</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
+          <t>$298-438</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Tasks/mês</t>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>LLM APIs</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>5.000</t>
+          <t>Flash+Sonnet+Opus via smart routing (MetaClaw)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>25.000</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>100.000+</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
+          <t>variável</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>$0.19/task</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>SLA</t>
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Cobrança cliente</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>99%</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>99.9%</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>99.95%</t>
-        </is>
-      </c>
+          <t>Mensalidade fixa + excedente por task</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>💰 Custos Nossos (USD)</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>POC (1 fundo)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>5K tasks/mês incluso</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>R$5.000/mês</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Infra EKS</t>
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Produção (5 fundos)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>$298</t>
+          <t>25K tasks/mês incluso</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>$438</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>$1.200+</t>
-        </is>
-      </c>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Control plane + nodes + RDS + networking</t>
+          <t>R$15.000/mês</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>LLM (smart routing)</t>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Enterprise (10+)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>$186</t>
+          <t>100K tasks, SLA 99.95%</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>$930</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>$3.720+</t>
-        </is>
-      </c>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Flash 60% + Sonnet 35% + Opus 5%</t>
+          <t>R$50.000/mês</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Suporte técnico</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>$500</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>$1.500</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Estimativa h/mês</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL CUSTO</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>$484</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>$1.868</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>$6.420+</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr"/>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>MARGEM SaaS</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>49-55% (sem BYOK) / 78-83% (com BYOK)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>✅ Recorrente</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>💵 Preço de Venda (BRL)</t>
+          <t>🅱 ON-PREM MAC MINI — Hardware dedicado no cliente</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Mensalidade sugerida</t>
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Descrição</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
+          <t>Mac Mini M4 Pro 64GB por colaborador/equipe. LLM local via Ollama/MLX.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Mac Mini M4 Pro 64GB + 1TB SSD</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>R$17.500</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>R$0</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Qwen 27B Q4: ~14 tok/s · Flash 8B: ~50 tok/s local</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>~R$0</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Energia</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>~40W TDP, 24/7</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>R$45/mês</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Suporte/licença</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Software Paganini + updates + suporte</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>R$2.000/mês</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Instalação, config, training da equipe (1-2 dias)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
           <t>R$5.000</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>R$15.000</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>R$50.000+</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Franquia inclusa (tasks)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>5.000</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>25.000</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>100.000</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Excedente por task</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>CAPEX total</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>1 Mac Mini + setup</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>R$22.500</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>OPEX total</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Licença + energia</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>R$2.045/mês</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>~R$0*</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Para 5 pessoas</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>5× Mac Mini + setup</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>R$112.500</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>R$10.225/mês</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>~R$0*</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>11 meses</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Para 10 pessoas</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>10× Mac Mini + setup</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>R$225.000</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>R$20.450/mês</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>~R$0*</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>11 meses</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>⚠ LIMITAÇÃO</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>LLM local (27B) é inferior a Sonnet/Opus. Bom para guardrails e triagem, ruim para análise complexa.</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr"/>
+      <c r="D23" s="9" t="inlineStr"/>
+      <c r="E23" s="9" t="inlineStr"/>
+      <c r="F23" s="9" t="inlineStr"/>
+      <c r="G23" s="9" t="inlineStr"/>
+      <c r="H23" s="9" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>🅲 PAY-PER-USE — Sem mensalidade, cobra por execução</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Zero compromisso. Cliente paga só quando usa. Preço por operação.</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Guardrail check</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Eligibility, concentration, covenant</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>R$0.25</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Classificação risco</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Risk scoring com Sonnet</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>R$0.80</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>R$0.80</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>R$0.50</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Acima da franquia</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Setup (one-time)</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Pipeline completo</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Todos os 6 guardrails + relatório</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>R$4.00</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Due Diligence</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Análise completa com Opus</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>R$5.00</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Volume 5K tasks/mês</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Equivalente ao POC SaaS</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>R$0</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>~R$5.750</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Volume 25K tasks/mês</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Equivalente à Produção</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>R$0</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>~R$28.750</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Desconto volume</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>10K+ = -15% · 50K+ = -25% · 100K+ = -35%</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>MARGEM Pay-per-Use</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>60-75%. Mais caro pro cliente em volume, mas zero risco de entrada.</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr"/>
+      <c r="D34" s="9" t="inlineStr"/>
+      <c r="E34" s="9" t="inlineStr"/>
+      <c r="F34" s="9" t="inlineStr"/>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>⚠ Receita variável</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>🅳 HÍBRIDO — Mac Mini local + Cloud API para tarefas pesadas</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Hardware local faz triagem/guardrails (custo ~R$0). Cloud APIs para análise complexa.</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Mac Mini (triagem)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Guardrails, RAG, classificação via LLM local</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>R$17.500</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>R$45/mês</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>~R$0</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr"/>
+      <c r="H38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>Cloud (análise)</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet/Opus para DD, compliance, decisão</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>variável</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>$0.19/task</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Mix estimado</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>70% local + 30% cloud → custo efetivo por task</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>R$0.30/task</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr"/>
+      <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Licença software</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Paganini + suporte + updates</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>R$3.000/mês</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>POC (1 fundo, 5K tasks)</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>1 Mac Mini + cloud overflow</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>R$22.500</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>R$3.350/mês</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>7 meses</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Produção (5 fundos, 25K)</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>3 Mac Mini + cloud overflow</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>R$67.500</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>R$10.900/mês</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>6 meses</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>VANTAGEM HÍBRIDO</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Menor custo operacional. Dados sensíveis processados local. Cloud só para LLM pesado.</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr"/>
+      <c r="D44" s="9" t="inlineStr"/>
+      <c r="E44" s="9" t="inlineStr"/>
+      <c r="F44" s="9" t="inlineStr"/>
+      <c r="G44" s="9" t="inlineStr"/>
+      <c r="H44" s="9" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>🅴 BYOK (Bring Your Own Keys) — Cliente paga LLM direto</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Cliente configura suas API keys (Anthropic, OpenAI, Google). Nós só cobramos plataforma.</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr"/>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>Infra (nós)</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>EKS compartilhado ou dedicado</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>$298-438</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>LLM (cliente)</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>API keys do cliente → custo variável é deles</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>$0 pra nós</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>$0 pra nós</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr"/>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>Licença plataforma</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr"/>
+      <c r="C50" s="3" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr"/>
+      <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>POC (1 fundo)</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Plataforma + suporte</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>R$3.500/mês</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Produção (5 fundos)</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Plataforma + suporte + SLA</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>R$10.500/mês</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>Enterprise (10+)</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated tenant + onboarding</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>R$37.500/mês</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Dia 1</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>Margem estimada</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Nosso custo = só infra (~R$1.500-2.300)</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr"/>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr"/>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>78-83%</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>VANTAGEM BYOK</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>Margem altíssima. Cliente controla custo de LLM. Compliance: dados passam pelas APIs deles.</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr"/>
+      <c r="D55" s="9" t="inlineStr"/>
+      <c r="E55" s="9" t="inlineStr"/>
+      <c r="F55" s="9" t="inlineStr"/>
+      <c r="G55" s="9" t="inlineStr"/>
+      <c r="H55" s="9" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>🅵 CONSULTORIA + LICENÇA — Implantação no ambiente do cliente</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Deployment no cloud/datacenter do cliente. Cobramos implantação + licença mensal.</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr"/>
+      <c r="F58" s="3" t="inlineStr"/>
+      <c r="G58" s="3" t="inlineStr"/>
+      <c r="H58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>Consultoria (setup)</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Arquitetura, deploy EKS/K8s, config, treinamento</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>R$50.000-150.000</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" s="3" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Licença mensal</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Software + updates + suporte L2/L3</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr"/>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>R$8.000-25.000</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr"/>
+      <c r="G60" s="3" t="inlineStr"/>
+      <c r="H60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>Infra (cliente)</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>AWS/Azure/GCP do próprio cliente</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>$0 pra nós</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>variável deles</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr"/>
+      <c r="G61" s="3" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>LLM (cliente)</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>API keys do cliente</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>$0 pra nós</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>variável deles</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr"/>
+      <c r="F62" s="3" t="inlineStr"/>
+      <c r="G62" s="3" t="inlineStr"/>
+      <c r="H62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>POC (1 fundo)</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Setup mínimo + 3 meses licença</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>R$50.000</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>R$8.000/mês</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr"/>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>1 projeto</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>Full deploy (10+)</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise setup + training</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>R$150.000</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>R$25.000/mês</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr"/>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>1 projeto</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>MARGEM CONSULTORIA</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>90%+ (nosso custo é tempo). Revenue mix: upfront + recorrente.</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr"/>
+      <c r="D65" s="9" t="inlineStr"/>
+      <c r="E65" s="9" t="inlineStr"/>
+      <c r="F65" s="9" t="inlineStr"/>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>✅ Melhor margem</t>
+        </is>
+      </c>
+      <c r="H65" s="9" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>📊 COMPARATIVO</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr"/>
+      <c r="C68" s="15" t="inlineStr"/>
+      <c r="D68" s="15" t="inlineStr"/>
+      <c r="E68" s="15" t="inlineStr"/>
+      <c r="F68" s="15" t="inlineStr"/>
+      <c r="G68" s="15" t="inlineStr"/>
+      <c r="H68" s="15" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: 1 fundo, 5.000 tasks/mês, 12 meses</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr"/>
+      <c r="C69" s="2" t="inlineStr"/>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>OPEX/mês</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>Custo ano 1</t>
+        </is>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>Custo ano 2</t>
+        </is>
+      </c>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t>Margem bruta</t>
+        </is>
+      </c>
+      <c r="G70" s="14" t="inlineStr">
+        <is>
+          <t>Melhor para</t>
+        </is>
+      </c>
+      <c r="H70" s="14" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>🅰 SaaS Cloud</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>R$0</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>R$5.000</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>R$15.000</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>R$60.000</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>R$120.000</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>49%</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Entrada rápida, zero CAPEX</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>🅱 On-Prem Mac Mini</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>R$22.500</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>R$2.045</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>R$47.040</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>R$71.580</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Privacidade, custos fixos</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>🅲 Pay-per-Use</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>R$0</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>~R$5.750</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>R$69.000</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>R$138.000</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Experimentação, volume variável</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>🅳 Híbrido</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>R$22.500</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>R$3.350</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>R$62.700</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>R$102.900</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>Equilíbrio custo × qualidade</t>
+        </is>
+      </c>
+      <c r="H74" s="18" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>🅴 BYOK Cloud</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>R$0</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>R$3.500</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>R$42.000</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>R$84.000</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>78%</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Compliance, cliente tech-savvy</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>🅵 Consultoria</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>R$50.000</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Onboarding + customização</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>📈 Margem</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Custo em BRL (@5.26)</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>R$2.546</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>R$9.826</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>R$33.769</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Receita</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>R$5.000</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>R$15.000</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>R$50.000</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Margem bruta</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>R$2.454</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>R$5.174</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>R$16.231</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Margem %</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>49%</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>34%</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>32%</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Antes de impostos</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>🔑 BYOK Discount</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Desconto se BYOK</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>-30%</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>-30%</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>-25%</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Cliente traz API keys</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Preço com BYOK</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>R$3.500</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>R$10.500</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>R$37.500</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Custo nosso com BYOK</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>R$1.568</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>R$2.304</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>R$6.312</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Só infra, sem LLM</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Margem com BYOK</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>55%</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>78%</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>83%</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Muito mais saudável</t>
-        </is>
-      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>R$8.000</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>R$146.000</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>R$242.000</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise, control total</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="19" t="inlineStr">
+        <is>
+          <t>💡 RECOMENDAÇÃO POC</t>
+        </is>
+      </c>
+      <c r="B78" s="19" t="inlineStr">
+        <is>
+          <t>Modelo 🅳 Híbrido para POC. Menor TCO 2 anos. Mac Mini local p/ triagem + Cloud para análise pesada. Escala para SaaS ou BYOK depois.</t>
+        </is>
+      </c>
+      <c r="C78" s="19" t="inlineStr"/>
+      <c r="D78" s="19" t="inlineStr"/>
+      <c r="E78" s="19" t="inlineStr"/>
+      <c r="F78" s="19" t="inlineStr"/>
+      <c r="G78" s="19" t="inlineStr"/>
+      <c r="H78" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4782,4 +6184,606 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dispositivo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CPU/GPU</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Preço BR</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Energia/mês</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>LLM 8B tok/s</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>LLM 27B tok/s</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Uso ideal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>🍎 Apple Silicon</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Mac Mini M4 16GB</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>M4 10-core, 10-core GPU</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>16GB UMA</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>R$7.500</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>R$30/mês</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>28-35 t/s</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>N/A (OOM)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Tarefas leves, 1 analista</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Mac Mini M4 24GB</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>M4 10-core, 10-core GPU</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>24GB UMA</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>R$9.000</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>R$30/mês</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>40-50 t/s</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>~5 t/s Q4</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Guardrails, triagem, RAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Mac Mini M4 Pro 48GB</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>M4 Pro 14-core, 20-core GPU</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>48GB UMA</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>R$14.000</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>R$40/mês</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>55+ t/s</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>11-14 t/s Q4</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Análise média, multi-user</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Mac Mini M4 Pro 64GB</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>M4 Pro 14-core, 20-core GPU</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>64GB UMA</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>R$17.500</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>R$45/mês</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>55+ t/s</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>14 t/s Q4</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>Recomendado POC ★</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Mac Studio M4 Max 128GB</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>M4 Max 16-core, 40-core GPU</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>128GB UMA</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>R$40.000</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>R$70/mês</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>100+ t/s</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>30+ t/s</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Server local, multi-tenant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>🟢 NVIDIA Edge</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Jetson Orin NX 16GB</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>8-core ARM, 157 TOPS</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>16GB</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>R$5.500</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>R$25/mês</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>15-20 t/s</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Edge, IoT, baixo consumo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Jetson AGX Orin 64GB</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>12-core ARM, 275 TOPS</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>64GB</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>R$15.000</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>R$45/mês</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>40+ t/s</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>~10 t/s</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Edge server, sem ventilação</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>☁️ Cloud GPU (referência)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>AWS g5.xlarge</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>A10G 24GB VRAM</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>16GB RAM</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>$1.006/h</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>~$750/mês</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>80+ t/s</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>25+ t/s</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Produção cloud, alta perf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>RunPod A100 80GB</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>A100 80GB VRAM</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>$1.19/h</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>~$857/mês</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>100+ t/s</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>37 t/s</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Training + inference</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>🖥 x86 Server (referência)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Dell PowerEdge + RTX 4090</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Xeon + RTX 4090 24GB</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>64GB DDR5</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>R$35.000</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>R$200/mês</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>80+ t/s</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>20+ t/s</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Datacenter on-prem</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Mini PC + RTX 4060 Ti</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>i7-14700 + 4060 Ti 16GB</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>32GB DDR5</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>R$12.000</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>R$100/mês</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>50+ t/s</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>~8 t/s Q4</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Budget on-prem</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>💡 PARA POC:</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Mac Mini M4 Pro 64GB é o sweet spot. R$17.500 por unidade. 14 tok/s no 27B local. Suficiente para guardrails + triagem. Análise pesada vai pra Cloud API.</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr"/>
+      <c r="D18" s="19" t="inlineStr"/>
+      <c r="E18" s="19" t="inlineStr"/>
+      <c r="F18" s="19" t="inlineStr"/>
+      <c r="G18" s="19" t="inlineStr"/>
+      <c r="H18" s="19" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: scaling curves sheet — 1 to 100 funds, infra thresholds, POC validation checklist
</commit_message>
<xml_diff>
--- a/packages/dashboard-v2/public/paganini-cost-model.xlsx
+++ b/packages/dashboard-v2/public/paganini-cost-model.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Modelos de Negócio" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Referências" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Hardware Specs" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Curva de Escala" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +91,16 @@
     <font>
       <b val="1"/>
       <color rgb="0016A34A"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00DC2626"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00DC2626"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -155,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,6 +190,14 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6786,4 +6805,2829 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I87"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>POC
+1 fundo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Seed
+3 fundos</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Growth
+10 fundos</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Scale
+25 fundos</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Enterprise
+50 fundos</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Mega
+100 fundos</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Economia
+de Escala</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Ação de Infra</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>📊 VOLUME DE OPERAÇÕES</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Tasks/mês</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>5.000</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>15.000</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>50.000</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>125.000</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>250.000</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>500.000</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Tasks/dia (avg)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1.667</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>4.167</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>8.333</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>16.667</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Tasks/hora (pico 3×)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>625</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>1.563</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>3.125</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>6.250</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Docs ingeridos/mês</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>5.000</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>12.500</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>25.000</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>50.000</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Usuários concorrentes</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>🖥 INFRA AWS (EKS) — o que muda a cada patamar</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>EKS Control Plane</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>$72</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>$72</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>$72</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>$72</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>$72</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>$72</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>Sempre 1 cluster (custo fixo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Worker Nodes</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>2× t3.medium
+$60</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>2× t3.medium
+$60</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>3× t3.large
+$180</t>
+        </is>
+      </c>
+      <c r="E11" s="22" t="inlineStr">
+        <is>
+          <t>4× t3.xlarge
+$480</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>6× t3.xlarge
+$720</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>8× t3.2xlarge
+$1.920</t>
+        </is>
+      </c>
+      <c r="H11" s="22" t="inlineStr">
+        <is>
+          <t>Escala ~linear</t>
+        </is>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>HPA auto-scaling por CPU/mem</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>RDS PostgreSQL</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>db.t3.medium
+$58</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>db.t3.medium
+$58</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>db.r6g.large
+$155</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>db.r6g.xlarge
+$310</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>db.r6g.2xlarge
+$620</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>db.r6g.4xlarge
+$1.240</t>
+        </is>
+      </c>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>Step function</t>
+        </is>
+      </c>
+      <c r="I12" s="22" t="inlineStr">
+        <is>
+          <t>Upgrade manual no threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>RDS Storage (pgvector)</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>50GB
+$6</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>100GB
+$12</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>250GB
+$30</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>500GB
+$60</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>1TB
+$120</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>2TB
+$240</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>Auto-grow habilitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>$22</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>$22</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>$22</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>$30</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>$40</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>$55</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>Sub-linear</t>
+        </is>
+      </c>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>LCU scaling automático</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>NAT Gateway</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>$46</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>$46</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>$60</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>$90</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>$130</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>$200</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>Sub-linear</t>
+        </is>
+      </c>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>2× para HA em produção</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>ElastiCache Redis</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>t3.medium
+$45</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>r6g.large
+$120</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>r6g.xlarge
+$240</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>r6g.2xlarge
+$480</t>
+        </is>
+      </c>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t>Step function</t>
+        </is>
+      </c>
+      <c r="I16" s="22" t="inlineStr">
+        <is>
+          <t>Cache para RAG + sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>S3 (corpus)</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>$3</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>$5</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>$25</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>$50</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I17" s="22" t="inlineStr">
+        <is>
+          <t>Docs + embeddings + backups</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>CloudWatch + logs</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>$20</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="inlineStr">
+        <is>
+          <t>$35</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>$60</t>
+        </is>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="G18" s="22" t="inlineStr">
+        <is>
+          <t>$180</t>
+        </is>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t>Sub-linear</t>
+        </is>
+      </c>
+      <c r="I18" s="22" t="inlineStr">
+        <is>
+          <t>Log retention 30d</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>WAF + Shield</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="G19" s="22" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="I19" s="22" t="inlineStr">
+        <is>
+          <t>DDoS + injection protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Data Transfer</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>$5</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>$30</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>$75</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>$150</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="inlineStr">
+        <is>
+          <t>$300</t>
+        </is>
+      </c>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I20" s="22" t="inlineStr">
+        <is>
+          <t>LLM API calls outbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL INFRA/mês</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>$287</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>$305</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>$654</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>$1.337</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>$2.257</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>$4.802</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>-52%/fundo</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>CUSTO INFRA/FUNDO</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>$287</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>$102</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>$65</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>$53</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>$45</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>$48</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>⬇ 83%</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Economia de escala real</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>🤖 LLM APIs — custo de tokens com smart routing</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Custo bruto (sem routing)</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>$930</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>$2.790</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>$9.300</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>$23.250</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>$46.500</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>$93.000</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I25" s="22" t="inlineStr">
+        <is>
+          <t>Modelo único Sonnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Smart routing MetaClaw</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr"/>
+      <c r="C26" s="22" t="inlineStr"/>
+      <c r="D26" s="22" t="inlineStr"/>
+      <c r="E26" s="22" t="inlineStr"/>
+      <c r="F26" s="22" t="inlineStr"/>
+      <c r="G26" s="22" t="inlineStr"/>
+      <c r="H26" s="22" t="inlineStr"/>
+      <c r="I26" s="22" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Flash (60% triagem)</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>$84</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>$252</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>$840</t>
+        </is>
+      </c>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>$2.100</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>$4.200</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="inlineStr">
+        <is>
+          <t>$8.400</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I27" s="22" t="inlineStr">
+        <is>
+          <t>$0.004/task</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sonnet (35% análise)</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>$665</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>$1.995</t>
+        </is>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>$6.650</t>
+        </is>
+      </c>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>$16.625</t>
+        </is>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>$33.250</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="inlineStr">
+        <is>
+          <t>$66.500</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I28" s="22" t="inlineStr">
+        <is>
+          <t>$0.038/task</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Opus (5% decisão)</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>$163</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>$488</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>$1.625</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>$4.063</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>$8.125</t>
+        </is>
+      </c>
+      <c r="G29" s="22" t="inlineStr">
+        <is>
+          <t>$16.250</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I29" s="22" t="inlineStr">
+        <is>
+          <t>$0.065/task</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Custo c/ routing</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>$912</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>$2.735</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>$9.115</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>$22.788</t>
+        </is>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>$45.575</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>$91.150</t>
+        </is>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>-2%</t>
+        </is>
+      </c>
+      <c r="I30" s="22" t="inlineStr">
+        <is>
+          <t>Saving modesto em routing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>Cache semântico (hit 30%)</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>-$274</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>-$821</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>-$2.735</t>
+        </is>
+      </c>
+      <c r="E31" s="22" t="inlineStr">
+        <is>
+          <t>-$6.836</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>-$13.673</t>
+        </is>
+      </c>
+      <c r="G31" s="22" t="inlineStr">
+        <is>
+          <t>-$27.345</t>
+        </is>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t>Sub-linear</t>
+        </is>
+      </c>
+      <c r="I31" s="22" t="inlineStr">
+        <is>
+          <t>Cache cresce com repetição</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Cache semântico (hit 60%)</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>-$547</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>-$1.641</t>
+        </is>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>-$5.469</t>
+        </is>
+      </c>
+      <c r="E32" s="22" t="inlineStr">
+        <is>
+          <t>-$13.673</t>
+        </is>
+      </c>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>-$27.345</t>
+        </is>
+      </c>
+      <c r="G32" s="22" t="inlineStr">
+        <is>
+          <t>-$54.690</t>
+        </is>
+      </c>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t>Sub-linear</t>
+        </is>
+      </c>
+      <c r="I32" s="22" t="inlineStr">
+        <is>
+          <t>Fundos similares = hit alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Batch processing (-15%)</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>-$96</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>-$287</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>-$957</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="inlineStr">
+        <is>
+          <t>-$2.393</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>-$4.785</t>
+        </is>
+      </c>
+      <c r="G33" s="22" t="inlineStr">
+        <is>
+          <t>-$9.573</t>
+        </is>
+      </c>
+      <c r="H33" s="22" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="I33" s="22" t="inlineStr">
+        <is>
+          <t>Não-urgentes em batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL LLM (cache 30%)</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>$1.627</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>$5.423</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>$13.559</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>$27.117</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>$54.232</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>-42% vs bruto</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>CUSTO LLM/FUNDO</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>Fixo/fundo</t>
+        </is>
+      </c>
+      <c r="I35" s="9" t="inlineStr">
+        <is>
+          <t>Escala LLM é linear por fundo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>💰 CUSTO TOTAL NOSSO (INFRA + LLM)</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Infra/mês</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>$287</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>$305</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>$654</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>$1.337</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>$2.257</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>$4.802</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>LLM/mês (cache 30%)</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>$542</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>$1.627</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>$5.423</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>$13.559</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>$27.117</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>$54.232</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Dev/Suporte (FTE parcial)</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>$1.500</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>$3.000</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>$5.000</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>$8.000</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>0.5-2 FTEs</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL/MÊS</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>$829</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>$2.432</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>$7.577</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>$17.896</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>$34.374</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>$67.034</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="inlineStr"/>
+      <c r="I41" s="15" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL/FUNDO/MÊS</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>$829</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>$811</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>$758</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>$716</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>$687</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>$670</t>
+        </is>
+      </c>
+      <c r="H42" s="15" t="inlineStr">
+        <is>
+          <t>⬇ 19%</t>
+        </is>
+      </c>
+      <c r="I42" s="15" t="inlineStr">
+        <is>
+          <t>Economia escala confirmada</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL/TASK</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>$0.166</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>$0.162</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>$0.152</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>$0.143</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>$0.137</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>$0.134</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>⬇ 19%</t>
+        </is>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>Custo unitário cai</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>💵 RECEITA (modelo SaaS, preço decrescente por volume)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>Preço/fundo/mês</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>R$5.000</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>R$4.500</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>R$3.500</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>R$3.000</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>R$2.500</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>R$2.000</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Desconto volume natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>Receita/mês (BRL)</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>R$5.000</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>R$13.500</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>R$35.000</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>R$75.000</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>R$125.000</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>R$200.000</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>Receita/mês (USD)</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>$950</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>$2.567</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>$6.654</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>$14.259</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>$23.764</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>$38.023</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>Custo/mês (USD)</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>$829</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>$2.432</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>$7.577</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>$17.896</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>$34.374</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>$67.034</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>Margem bruta (USD)</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>$121</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>$135</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>-$923</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>-$3.637</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>-$10.610</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>-$29.011</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>Margem %</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="D51" s="23" t="inlineStr">
+        <is>
+          <t>-14%</t>
+        </is>
+      </c>
+      <c r="E51" s="23" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="F51" s="23" t="inlineStr">
+        <is>
+          <t>-45%</t>
+        </is>
+      </c>
+      <c r="G51" s="23" t="inlineStr">
+        <is>
+          <t>-76%</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Preço baixo demais</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="inlineStr">
+        <is>
+          <t>⚠ INSIGHT CRÍTICO</t>
+        </is>
+      </c>
+      <c r="B53" s="24" t="inlineStr">
+        <is>
+          <t>LLM escala LINEAR por fundo. Infra escala sub-linear. Mas LLM domina 65-92% do custo. Sem cache agressivo ou BYOK, escala grande é DEFICITÁRIA com preço decrescente.</t>
+        </is>
+      </c>
+      <c r="C53" s="24" t="inlineStr"/>
+      <c r="D53" s="24" t="inlineStr"/>
+      <c r="E53" s="24" t="inlineStr"/>
+      <c r="F53" s="24" t="inlineStr"/>
+      <c r="G53" s="24" t="inlineStr"/>
+      <c r="H53" s="24" t="inlineStr"/>
+      <c r="I53" s="24" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>✅ ESCALA SAUDÁVEL — modelo BYOK (cliente paga LLM)</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>Custo nosso (só infra)</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>$287</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>$305</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>$654</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>$1.337</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>$2.257</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>$4.802</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Zero LLM no nosso P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>Preço BYOK/fundo/mês</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>R$3.500</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>R$3.000</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>R$2.500</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>R$2.000</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>R$1.800</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>R$1.500</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Mais barato pro cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>Receita/mês (USD)</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>$665</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>$1.711</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>$4.753</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>$9.506</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>$17.110</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>$28.517</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>Margem bruta (USD)</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>$378</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>$1.406</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>$4.099</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>$8.169</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>$14.853</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>$23.715</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr"/>
+      <c r="I59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Margem %</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>82%</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
+        <is>
+          <t>86%</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>86%</t>
+        </is>
+      </c>
+      <c r="F60" s="20" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="G60" s="20" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr"/>
+      <c r="I60" s="20" t="inlineStr">
+        <is>
+          <t>✅ Escala saudável</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="19" t="inlineStr">
+        <is>
+          <t>✅ CONCLUSÃO ESCALA</t>
+        </is>
+      </c>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>Para validar escala na POC, o modelo BYOK ou Híbrido é obrigatório. SaaS puro com LLM nosso não escala acima de 5 fundos sem margem negativa. A POC deve testar: 1) cache semântico, 2) routing MetaClaw, 3) throughput por nó, 4) latência P95 sob carga.</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="inlineStr"/>
+      <c r="D62" s="19" t="inlineStr"/>
+      <c r="E62" s="19" t="inlineStr"/>
+      <c r="F62" s="19" t="inlineStr"/>
+      <c r="G62" s="19" t="inlineStr"/>
+      <c r="H62" s="19" t="inlineStr"/>
+      <c r="I62" s="19" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>🔧 THRESHOLDS DE ESCALA — quando fazer upgrade</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" s="2" t="inlineStr"/>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>De</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Para</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Custo adicional</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Downtime</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>CPU &gt; 70% sustained</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Add worker node</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>2 nodes</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>3 nodes</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>+$30/mês</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Zero (rolling)</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>RAM &gt; 80%</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade node type</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>t3.medium</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>t3.large</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>+$60/mês</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>~2min (drain+replace)</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr"/>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>DB connections &gt; 80%</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade RDS</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>db.t3.medium</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>db.r6g.large</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>+$97/mês</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>~5min (failover)</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr"/>
+      <c r="H68" s="3" t="inlineStr"/>
+      <c r="I68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>pgvector &gt; 500K rows</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Add IVFFlat index</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Index rebuild</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>~0 (compute)</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Zero</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr"/>
+      <c r="H69" s="3" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>Cache miss &gt; 50%</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Add ElastiCache</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>t3.medium Redis</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>+$45/mês</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Zero</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr"/>
+      <c r="H70" s="3" t="inlineStr"/>
+      <c r="I70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>Latência P95 &gt; 5s</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Add Sonnet replica</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>1 region</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>2 regions</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>+$50/mês (ALB)</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Zero</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr"/>
+      <c r="H71" s="3" t="inlineStr"/>
+      <c r="I71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
+        <is>
+          <t>Tasks/h &gt; 1.000</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Enable batch queue</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Sync</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>SQS + async</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>~$5/mês</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Zero</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr"/>
+      <c r="H72" s="3" t="inlineStr"/>
+      <c r="I72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>Fundos &gt; 25</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Multi-AZ mandatory</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Single-AZ</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Multi-AZ RDS</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>+$155/mês</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>~5min</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr"/>
+      <c r="H73" s="3" t="inlineStr"/>
+      <c r="I73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>Fundos &gt; 50</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated EKS</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Shared cluster</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Client cluster</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>+$72/mês</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr"/>
+      <c r="H74" s="3" t="inlineStr"/>
+      <c r="I74" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="15" t="inlineStr">
+        <is>
+          <t>📋 CHECKLIST DE VALIDAÇÃO NA POC</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="inlineStr"/>
+      <c r="C77" s="15" t="inlineStr"/>
+      <c r="D77" s="15" t="inlineStr"/>
+      <c r="E77" s="15" t="inlineStr"/>
+      <c r="F77" s="15" t="inlineStr"/>
+      <c r="G77" s="15" t="inlineStr"/>
+      <c r="H77" s="15" t="inlineStr"/>
+      <c r="I77" s="15" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t>1. Throughput</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Processar 100 tasks em 10 min (10 tasks/min sustentado)</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Meta: &gt;167 tasks/dia</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr"/>
+      <c r="E78" s="3" t="inlineStr"/>
+      <c r="F78" s="3" t="inlineStr"/>
+      <c r="G78" s="3" t="inlineStr"/>
+      <c r="H78" s="3" t="inlineStr"/>
+      <c r="I78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t>2. Latência P95</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Pipeline completo &lt; 8 segundos em P95</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Meta: &lt;5s avg</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr"/>
+      <c r="F79" s="3" t="inlineStr"/>
+      <c r="G79" s="3" t="inlineStr"/>
+      <c r="H79" s="3" t="inlineStr"/>
+      <c r="I79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="inlineStr">
+        <is>
+          <t>3. Cache hit rate</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Medir taxa de cache semântico com corpus real do fundo</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Meta: &gt;30% hit</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr"/>
+      <c r="E80" s="3" t="inlineStr"/>
+      <c r="F80" s="3" t="inlineStr"/>
+      <c r="G80" s="3" t="inlineStr"/>
+      <c r="H80" s="3" t="inlineStr"/>
+      <c r="I80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t>4. Concurrent users</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>5 usuários simultâneos sem degradação &gt;20%</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Meta: &lt;6s P95</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr"/>
+      <c r="E81" s="3" t="inlineStr"/>
+      <c r="F81" s="3" t="inlineStr"/>
+      <c r="G81" s="3" t="inlineStr"/>
+      <c r="H81" s="3" t="inlineStr"/>
+      <c r="I81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t>5. Smart routing</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar que MetaClaw usa Flash para 60%+ das tasks</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Meta: &gt;55% Flash</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr"/>
+      <c r="E82" s="3" t="inlineStr"/>
+      <c r="F82" s="3" t="inlineStr"/>
+      <c r="G82" s="3" t="inlineStr"/>
+      <c r="H82" s="3" t="inlineStr"/>
+      <c r="I82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t>6. Accuracy</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Guardrails concordam com analista humano em 90%+ dos casos</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Meta: &gt;90%</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr"/>
+      <c r="E83" s="3" t="inlineStr"/>
+      <c r="F83" s="3" t="inlineStr"/>
+      <c r="G83" s="3" t="inlineStr"/>
+      <c r="H83" s="3" t="inlineStr"/>
+      <c r="I83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>7. Cost tracking</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Medir custo real por task vs estimativa da planilha</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Meta: ±20%</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr"/>
+      <c r="E84" s="3" t="inlineStr"/>
+      <c r="F84" s="3" t="inlineStr"/>
+      <c r="G84" s="3" t="inlineStr"/>
+      <c r="H84" s="3" t="inlineStr"/>
+      <c r="I84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>8. Horizontal scale</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Adicionar 2º worker node sob carga, medir melhoria</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Meta: ~linear</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr"/>
+      <c r="E85" s="3" t="inlineStr"/>
+      <c r="F85" s="3" t="inlineStr"/>
+      <c r="G85" s="3" t="inlineStr"/>
+      <c r="H85" s="3" t="inlineStr"/>
+      <c r="I85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>9. Failover</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Matar 1 worker node, confirmar recuperação automática</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Meta: &lt;60s</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr"/>
+      <c r="E86" s="3" t="inlineStr"/>
+      <c r="F86" s="3" t="inlineStr"/>
+      <c r="G86" s="3" t="inlineStr"/>
+      <c r="H86" s="3" t="inlineStr"/>
+      <c r="I86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>10. Data isolation</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar que fundo A não vê dados do fundo B</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Meta: 100%</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="3" t="inlineStr"/>
+      <c r="G87" s="3" t="inlineStr"/>
+      <c r="H87" s="3" t="inlineStr"/>
+      <c r="I87" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: unified infra sheet — EC2 standalone (atual + otimizada + RI) vs EKS (POC + prod) with comparison
</commit_message>
<xml_diff>
--- a/packages/dashboard-v2/public/paganini-cost-model.xlsx
+++ b/packages/dashboard-v2/public/paganini-cost-model.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Infra EKS - POC" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Infra — EC2 + EKS" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tokens &amp; Tarefas" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Tech Stack Atual" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Retroativo (32 dias)" sheetId="4" state="visible" r:id="rId4"/>
@@ -28,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,6 +102,12 @@
       <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
+    <font>
+      <color rgb="00DC2626"/>
+    </font>
+    <font>
+      <color rgb="0016A34A"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -166,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -198,6 +204,8 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,16 +571,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -609,7 +617,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>% Total</t>
+          <t>Tipo custo</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -619,225 +627,237 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>🎛 Control Plane</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>OPÇÃO A: EC2 STANDALONE</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Infra atual — deploy direto, sem orquestração K8s</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr"/>
+      <c r="D2" s="15" t="inlineStr"/>
+      <c r="E2" s="15" t="inlineStr"/>
+      <c r="F2" s="15" t="inlineStr"/>
+      <c r="G2" s="15" t="inlineStr"/>
+      <c r="H2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>EKS Cluster</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Managed K8s 1.31, standard support</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>🖥 EC2 — Setup Atual (em produção hoje)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>EC2 openclaw (ATUAL)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>t2.2xlarge · 8 vCPU · 32GB · sa-east-1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>72</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>379</v>
-      </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Custo fixo por cluster</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>🖥 Compute (Node Group)</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="D4" s="3" t="n">
+        <v>0.3712</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>267</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>1404</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>⚠ OVERSIZED — usa ~1GB de 32GB</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>EC2 t3.medium</t>
+          <t>EC2 aios-paganini (ATUAL)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2 vCPU, 4GB RAM, multi-AZ</t>
+          <t>t2.2xlarge · 8 vCPU · 32GB · DESLIGADA</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>0.0416</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>316</v>
-      </c>
-      <c r="G5" s="3" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.3712</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Stopped</t>
+        </is>
+      </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>On-Demand. Spot = -60%</t>
+          <t>✅ Desligada 25/Mar</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>EBS gp3 50GB</t>
+          <t>EBS gp3 (openclaw)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Root volumes worker nodes</t>
+          <t>40GB root volume</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="3" t="n"/>
-      <c r="E6" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>42</v>
-      </c>
-      <c r="G6" s="3" t="n"/>
+      <c r="E6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>3000 IOPS included</t>
+          <t>Inclui Docker + pgvector</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>🗄 Database</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>EBS gp3 (paganini)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>40GB root volume</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Storage enquanto stopped</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>RDS PostgreSQL</t>
+          <t>Elastic IP</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>db.t3.medium, pgvector, Single-AZ</t>
+          <t>IP público fixo</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="5" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>305</v>
-      </c>
-      <c r="G8" s="3" t="n"/>
+      <c r="D8" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Multi-AZ = 2× custo</t>
+          <t>$0.005/h se associado</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>RDS Storage gp3</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>50GB para embeddings + state</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Cresce ~2GB/mês</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>RDS Backups</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Daily automated, 7d retention</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Incluso até 100% do storage</t>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL EC2 (ATUAL)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Custo real hoje (com paganini desligada)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>$278</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>R$1.462</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>97% RAM desperdiçada</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>🌐 Networking</t>
+          <t>🖥 EC2 — POC OTIMIZADA (recomendado)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
@@ -851,375 +871,1606 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ALB</t>
+          <t>EC2 Paganini API</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Application Load Balancer, HTTPS</t>
+          <t>t3.small · 2 vCPU · 2GB · sa-east-1</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="5" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>116</v>
-      </c>
-      <c r="G12" s="3" t="n"/>
+      <c r="D12" s="3" t="n">
+        <v>0.0208</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Path routing, health checks</t>
+          <t>Docker + FastAPI + Paganini serve</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>NAT Gateway</t>
+          <t>EC2 Gateway OpenClaw</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Outbound para LLM APIs</t>
+          <t>t3.small · 2 vCPU · 2GB · sa-east-1</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="5" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>195</v>
-      </c>
-      <c r="G13" s="3" t="n"/>
+      <c r="D13" s="3" t="n">
+        <v>0.0208</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>Prod: 2× para HA</t>
+          <t>Gateway + pgvector container</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>NAT Data Processing</t>
+          <t>EBS gp3 (Paganini)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>~200GB/mês estimado</t>
+          <t>30GB root + 20GB data</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="3" t="n"/>
-      <c r="E14" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>47</v>
-      </c>
-      <c r="G14" s="3" t="n"/>
+      <c r="E14" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>$0.045/GB processado</t>
+          <t>Corpus docs + embeddings</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Public IPv4</t>
+          <t>EBS gp3 (Gateway)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ALB + NAT Gateway</t>
+          <t>20GB root</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="5" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>37</v>
-      </c>
-      <c r="G15" s="3" t="n"/>
+      <c r="F15" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>$0.005/h por IP</t>
+          <t>Minimal</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>📦 Storage &amp; Monitoring</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>RDS PostgreSQL</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>db.t3.micro · 2 vCPU · 1GB · pgvector</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Free tier eligible (750h/mês)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>RDS Storage gp3</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Corpus docs + DB snapshots (~10GB)</t>
+          <t>20GB inicial</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="3" t="n"/>
-      <c r="E17" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="G17" s="3" t="n"/>
+      <c r="E17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>$0.023/GB/mês</t>
+          <t>Auto-grow</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>CloudWatch</t>
+          <t>Elastic IP × 2</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Logs, métricas, alarms</t>
+          <t>IPs públicos fixos</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="G18" s="3" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Basic monitoring</t>
+          <t>1 por instância</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>ECR</t>
+          <t>Data Transfer</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Container registry (~5GB)</t>
+          <t>~50GB outbound/mês</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="3" t="n"/>
-      <c r="E19" s="6" t="n">
+      <c r="E19" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>$0.09/GB após 1GB free</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>CloudWatch Basic</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Métricas + 2 alarms</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="7" t="n">
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="F20" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>CPU, disk, memory alarms</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>S3 (backups)</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>10GB DB snapshots + docs</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>$0.023/GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL EC2 POC</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>2× t3.small + RDS micro + storage</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr"/>
+      <c r="D22" s="9" t="inlineStr"/>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>$71</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>R$374</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr"/>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Saving 74% vs atual</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>🖥 EC2 — POC COM RESERVA 1 ANO (saving adicional)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>EC2 t3.small RI 1Y</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>All Upfront 1 ano (2 instâncias)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Saving 42% vs On-Demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>RDS t3.micro RI 1Y</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>All Upfront 1 ano</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Saving 41%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL EC2 RI</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Com reserva 1 ano (upfront ~$300)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr"/>
+      <c r="D26" s="9" t="inlineStr"/>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>$46</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>R$242</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr"/>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Saving 83% vs atual</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>OPÇÃO B: EKS KUBERNETES</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Orquestração containerizada — escala horizontal automática</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr"/>
+      <c r="D29" s="15" t="inlineStr"/>
+      <c r="E29" s="15" t="inlineStr"/>
+      <c r="F29" s="15" t="inlineStr"/>
+      <c r="G29" s="15" t="inlineStr"/>
+      <c r="H29" s="15" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>🎛 Control Plane</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>EKS Cluster</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Managed K8s 1.31, standard support</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>Custo fixo por cluster</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>🖥 Compute (Node Group)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>EC2 t3.medium (workers)</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>2 vCPU, 4GB RAM, multi-AZ</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0.0416</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>316</v>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>Spot = -60%. HPA auto-scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>EBS gp3 50GB</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Root volumes worker nodes</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>3000 IOPS included</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>🗄 Database</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>RDS PostgreSQL</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>db.t3.medium, pgvector, Single-AZ</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>305</v>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Multi-AZ = 2× custo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>RDS Storage gp3</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>50GB para embeddings + state</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Cresce ~2GB/mês</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>RDS Backups</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Daily automated, 7d retention</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="3" t="n"/>
+      <c r="E38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Incluso</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Incluso até 100% do storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>🌐 Networking</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Application Load Balancer, HTTPS</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Path routing, health checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>NAT Gateway</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Outbound para LLM APIs</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>Prod: 2× para HA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>NAT Data Processing</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>~200GB/mês estimado</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>$0.045/GB processado</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Public IPv4</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>ALB + NAT Gateway</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>$0.005/h por IP</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>📦 Storage &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Corpus docs + DB snapshots (~10GB)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>$0.023/GB/mês</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>CloudWatch</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Logs, métricas, alarms</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Basic monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>ECR</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Container registry (~5GB)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="3" t="n"/>
+      <c r="E47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
         <is>
           <t>$0.10/GB/mês</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>SUBTOTAL INFRA POC</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n">
-        <v>298</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1568</v>
-      </c>
-      <c r="G20" s="9" t="inlineStr"/>
-      <c r="H20" s="9" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>UPGRADES PARA PRODUÇÃO</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL EKS POC</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Cluster + 2 workers + RDS + ALB + NAT</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr"/>
+      <c r="D48" s="9" t="inlineStr"/>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>$298</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>R$1.568</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr"/>
+      <c r="H48" s="9" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>⬆️ Upgrades para EKS Produção</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Node Group → 3 nodes</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>HA cross-AZ</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>+$30</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>+R$158</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="C51" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>158</v>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>Auto-scaling 2-5 nodes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>RDS Multi-AZ</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>Standby + failover automático</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>+$58</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>+R$305</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="C52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="3" t="n"/>
+      <c r="E52" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>305</v>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>Uptime SLA 99.95%</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>NAT Gateway × 2</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>HA networking</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>+$37</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>+R$195</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="C53" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="3" t="n"/>
+      <c r="E53" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>On-Demand</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>1 por AZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>WAF</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Firewall, DDoS, injection protection</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>+$10</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>+R$53</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="C54" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H54" s="8" t="inlineStr">
+        <is>
+          <t>Web ACL + managed rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Secrets Manager</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Rotação automática de keys</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>+$5</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>+R$26</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>SUBTOTAL PROD</t>
-        </is>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>Infra total produção</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
+      <c r="C55" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Fixo</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>$0.40/secret/mês</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL EKS PROD</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>Tudo acima + upgrades HA</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr"/>
+      <c r="D56" s="9" t="inlineStr"/>
+      <c r="E56" s="9" t="inlineStr">
         <is>
           <t>$438</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F56" s="9" t="inlineStr">
         <is>
           <t>R$2.304</t>
         </is>
       </c>
+      <c r="G56" s="9" t="inlineStr"/>
+      <c r="H56" s="9" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>📊 COMPARATIVO EC2 vs EKS</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr"/>
+      <c r="C59" s="15" t="inlineStr"/>
+      <c r="D59" s="15" t="inlineStr"/>
+      <c r="E59" s="15" t="inlineStr"/>
+      <c r="F59" s="15" t="inlineStr"/>
+      <c r="G59" s="15" t="inlineStr"/>
+      <c r="H59" s="15" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Critério</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>EC2 Standalone (POC)</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>EC2 com RI 1Y</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>EKS POC</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
+          <t>EKS Prod</t>
+        </is>
+      </c>
+      <c r="F60" s="14" t="inlineStr"/>
+      <c r="G60" s="14" t="inlineStr"/>
+      <c r="H60" s="14" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>Custo/mês</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>$71</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>$46</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>$298</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>$438</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr"/>
+      <c r="G61" s="3" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>Custo/mês (BRL)</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>R$374</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>R$242</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>R$1.568</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>R$2.304</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr"/>
+      <c r="G62" s="3" t="inlineStr"/>
+      <c r="H62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>Setup time</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>2-4 horas</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>2-4h + reserva</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>1-2 dias</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>2-3 dias</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr"/>
+      <c r="G63" s="3" t="inlineStr"/>
+      <c r="H63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>Auto-scaling</t>
+        </is>
+      </c>
+      <c r="B64" s="25" t="inlineStr">
+        <is>
+          <t>❌ Manual</t>
+        </is>
+      </c>
+      <c r="C64" s="25" t="inlineStr">
+        <is>
+          <t>❌ Manual</t>
+        </is>
+      </c>
+      <c r="D64" s="26" t="inlineStr">
+        <is>
+          <t>✅ HPA/VPA</t>
+        </is>
+      </c>
+      <c r="E64" s="26" t="inlineStr">
+        <is>
+          <t>✅ HPA/VPA + Cluster</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr"/>
+      <c r="G64" s="3" t="inlineStr"/>
+      <c r="H64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>Rolling deploy</t>
+        </is>
+      </c>
+      <c r="B65" s="25" t="inlineStr">
+        <is>
+          <t>❌ Downtime</t>
+        </is>
+      </c>
+      <c r="C65" s="25" t="inlineStr">
+        <is>
+          <t>❌ Downtime</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>✅ Zero-downtime</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="inlineStr">
+        <is>
+          <t>✅ Blue/Green</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr"/>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>Multi-AZ / HA</t>
+        </is>
+      </c>
+      <c r="B66" s="25" t="inlineStr">
+        <is>
+          <t>❌ Single-AZ</t>
+        </is>
+      </c>
+      <c r="C66" s="25" t="inlineStr">
+        <is>
+          <t>❌ Single-AZ</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Parcial</t>
+        </is>
+      </c>
+      <c r="E66" s="26" t="inlineStr">
+        <is>
+          <t>✅ Full HA</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr"/>
+      <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>Load balancing</t>
+        </is>
+      </c>
+      <c r="B67" s="25" t="inlineStr">
+        <is>
+          <t>❌ Nginx manual</t>
+        </is>
+      </c>
+      <c r="C67" s="25" t="inlineStr">
+        <is>
+          <t>❌ Nginx manual</t>
+        </is>
+      </c>
+      <c r="D67" s="26" t="inlineStr">
+        <is>
+          <t>✅ ALB nativo</t>
+        </is>
+      </c>
+      <c r="E67" s="26" t="inlineStr">
+        <is>
+          <t>✅ ALB + WAF</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr"/>
+      <c r="G67" s="3" t="inlineStr"/>
+      <c r="H67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>Max fundos (confortável)</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>3-10</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>10-100+</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr"/>
+      <c r="G68" s="3" t="inlineStr"/>
+      <c r="H68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>Migração para prod</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Requer refactor</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Requer refactor</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Escala in-place</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Já é prod</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr"/>
+      <c r="G69" s="3" t="inlineStr"/>
+      <c r="H69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>Complexidade ops</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Baixa</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Baixa</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>🟡 Média</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>🟡 Média</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr"/>
+      <c r="G70" s="3" t="inlineStr"/>
+      <c r="H70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>Ideal para</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>POC rápida, 1 fundo</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>POC 6-12 meses</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Validar escala</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Produção real</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr"/>
+      <c r="G71" s="3" t="inlineStr"/>
+      <c r="H71" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="19" t="inlineStr">
+        <is>
+          <t>💡 RECOMENDAÇÃO</t>
+        </is>
+      </c>
+      <c r="B73" s="19" t="inlineStr">
+        <is>
+          <t>POC começa em EC2 ($71/mês). Valida produto com 1 fundo. Quando escalar para 3+ fundos, migra para EKS ($298/mês). EKS valida auto-scaling e HA — o que o cliente quer ver.</t>
+        </is>
+      </c>
+      <c r="C73" s="19" t="inlineStr"/>
+      <c r="D73" s="19" t="inlineStr"/>
+      <c r="E73" s="19" t="inlineStr"/>
+      <c r="F73" s="19" t="inlineStr"/>
+      <c r="G73" s="19" t="inlineStr"/>
+      <c r="H73" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: Linear 8/mês (Standard), not free
</commit_message>
<xml_diff>
--- a/packages/dashboard-v2/public/paganini-cost-model.xlsx
+++ b/packages/dashboard-v2/public/paganini-cost-model.xlsx
@@ -3451,23 +3451,23 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Review hub.</t>
+          <t>Review hub + project management.</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.1%</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -3642,10 +3642,10 @@
       <c r="B21" s="15" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n">
-        <v>860</v>
+        <v>878</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>4524</v>
+        <v>4619</v>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: full license & compliance audit — 112 deps, 98% permissive, 0 GPL
</commit_message>
<xml_diff>
--- a/packages/dashboard-v2/public/paganini-cost-model.xlsx
+++ b/packages/dashboard-v2/public/paganini-cost-model.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Referências" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Hardware Specs" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Curva de Escala" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Licenças &amp; Compliance" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,6 +109,10 @@
     <font>
       <color rgb="0016A34A"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -172,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -206,6 +211,8 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2477,6 +2484,2944 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H92"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Versão</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Licença</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Comercial?</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Obrigação</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>🔵 CÓDIGO PRÓPRIO PAGANINI</t>
+        </is>
+      </c>
+      <c r="B2" s="27" t="inlineStr"/>
+      <c r="C2" s="27" t="inlineStr"/>
+      <c r="D2" s="27" t="inlineStr"/>
+      <c r="E2" s="27" t="inlineStr"/>
+      <c r="F2" s="27" t="inlineStr"/>
+      <c r="G2" s="27" t="inlineStr"/>
+      <c r="H2" s="27" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>paganini-aios (backend)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Próprio</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>✅ Total</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Zero</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma — nosso IP</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>40 .py, 7.2K LOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>paganini-dashboard-v2</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2.0.0</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Proprietário</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Próprio</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>✅ Total</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Zero</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma — nosso IP</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Next.js frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>MetaClaw (smart routing)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Proprietário</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Próprio</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>✅ Total</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Zero</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma — nosso IP</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Moltis (kernel runtime)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Proprietário</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Próprio</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>✅ Total</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Zero</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma — nosso IP</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Agent orchestration core</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>9 agentes FIDC</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Proprietário</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Próprio</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>✅ Total</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Zero</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma — nosso IP</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Guardrails, compliance, DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Hybrid RAG pipeline</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Proprietário</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Próprio</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>✅ Total</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Zero</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma — nosso IP</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Dense+sparse+graph→RRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>🐍 DEPENDÊNCIAS PYTHON (runtime)</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr"/>
+      <c r="C10" s="27" t="inlineStr"/>
+      <c r="D10" s="27" t="inlineStr"/>
+      <c r="E10" s="27" t="inlineStr"/>
+      <c r="F10" s="27" t="inlineStr"/>
+      <c r="G10" s="27" t="inlineStr"/>
+      <c r="H10" s="27" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>✅ Licenças Permissivas (MIT / BSD / Apache) — sem restrição comercial</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>LiteLLM</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=1.0</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Gateway para 100+ LLMs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>FastAPI</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=0.115</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>API framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Uvicorn</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=0.32</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>BSD-3-Clause</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>ASGI server</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Pydantic</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=2.0</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Data validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Click</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=8.0</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>BSD-3-Clause</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>CLI framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Rich</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=13.0</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Terminal formatting</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>PyYAML</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=6.0</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>YAML parser</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>HTTPX</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=0.27</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>BSD-3-Clause</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright no LICENSE</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>HTTP client</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ChromaDB</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=1.0</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright + NOTICE</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Vector store (embedded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Hatchling</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma (build-time only)</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Não vai pro deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>⚠️ Dependências opcionais [rl] — só para treinamento, NÃO vai pro produto</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>PyTorch</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=2.0</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>BSD-3-Clause</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>ML Framework</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Só para SFT/GRPO training</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Transformers</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=4.40</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>ML Framework</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright + NOTICE</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>HuggingFace. Só training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Pytest</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>&gt;=7.0</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma (dev-only)</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Não vai pro deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Ruff / Black / isort</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Lint/Format</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma (dev-only)</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Não vai pro deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="27" t="inlineStr">
+        <is>
+          <t>📦 DEPENDÊNCIAS JAVASCRIPT (dashboard)</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr"/>
+      <c r="C28" s="27" t="inlineStr"/>
+      <c r="D28" s="27" t="inlineStr"/>
+      <c r="E28" s="27" t="inlineStr"/>
+      <c r="F28" s="27" t="inlineStr"/>
+      <c r="G28" s="27" t="inlineStr"/>
+      <c r="H28" s="27" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>✅ Licenças Permissivas — 109 de 112 pacotes</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Next.js</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>^15.0</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>React meta-framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>React / React-DOM</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>^19.0</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>UI library</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Supabase JS</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>^2.100</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>DB client</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Tailwind CSS</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>^4.2</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Utility CSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Recharts</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>^2.15</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Chart library</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Three.js</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>^0.183</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>3D rendering</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>react-force-graph-3d</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>^1.29</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Graph visualization</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Lucide React</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>^0.468</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>ISC</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Icons</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Incluir copyright</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Icon set</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>TypeScript</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma (dev-only)</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Não vai pro deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>PostCSS</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>^8.5</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma (build-only)</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>CSS processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>+ 99 transitivas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>MIT/ISC/BSD</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Deps</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Automático via bundler</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Todas permissivas</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>⚠️ LGPL — 2 pacotes (sharp/libvips)</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>@img/sharp-libvips-linux-x64</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>1.2.4</t>
+        </is>
+      </c>
+      <c r="C42" s="28" t="inlineStr">
+        <is>
+          <t>LGPL-3.0</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Dep transitiva</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Condicional</t>
+        </is>
+      </c>
+      <c r="F42" s="28" t="inlineStr">
+        <is>
+          <t>🟡 Médio</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Não modificar. Link dinâmico OK.</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Usado por Next.js Image Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>@img/sharp-libvips-linuxmusl</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>1.2.4</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="inlineStr">
+        <is>
+          <t>LGPL-3.0</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Dep transitiva</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Condicional</t>
+        </is>
+      </c>
+      <c r="F43" s="28" t="inlineStr">
+        <is>
+          <t>🟡 Médio</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Não modificar. Link dinâmico OK.</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Idem — variant musl</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>☁️ INFRAESTRUTURA &amp; SERVIÇOS EXTERNOS</t>
+        </is>
+      </c>
+      <c r="B45" s="27" t="inlineStr"/>
+      <c r="C45" s="27" t="inlineStr"/>
+      <c r="D45" s="27" t="inlineStr"/>
+      <c r="E45" s="27" t="inlineStr"/>
+      <c r="F45" s="27" t="inlineStr"/>
+      <c r="G45" s="27" t="inlineStr"/>
+      <c r="H45" s="27" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Cloud &amp; SaaS — contratos de uso, não licenças de código</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>AWS (EC2/EKS/RDS/S3)</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>AWS ToS</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>IaaS</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Pagar pelo uso. Sem lock-in de IP.</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Multi-region disponível</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0 (OSS)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>BaaS</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Self-host possível. Sem vendor lock.</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>OSS core, hosted service</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Vercel ToS</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>PaaS</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Pagar pelo uso. Migrar pra Cloudflare se quiser.</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Deploy frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Docker</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Runtime</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Docker Engine é OSS.</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Container runtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes / Helm</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Orchestration</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>CNCF project, totalmente aberto.</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Container orchestration</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>PostgreSQL License</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Mais permissiva que MIT.</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>DB engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>pgvector</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>0.7+</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>PostgreSQL License</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Extension</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Mais permissiva que MIT.</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Vector similarity</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Nginx</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>BSD-2-Clause</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma restrição.</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Reverse proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Cloudflare Tunnel</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Cloudflare ToS</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Free tier. Pagar se escalar.</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Zero-trust tunnels</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="27" t="inlineStr">
+        <is>
+          <t>🤖 LLM APIs — TERMS OF SERVICE CRÍTICOS</t>
+        </is>
+      </c>
+      <c r="B57" s="27" t="inlineStr"/>
+      <c r="C57" s="27" t="inlineStr"/>
+      <c r="D57" s="27" t="inlineStr"/>
+      <c r="E57" s="27" t="inlineStr"/>
+      <c r="F57" s="27" t="inlineStr"/>
+      <c r="G57" s="27" t="inlineStr"/>
+      <c r="H57" s="27" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Provedores de API — pagar por token, sem licença de modelo</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic Claude API</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet/Opus</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic ToS</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Output não pode treinar modelos concorrentes.</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Comercial OK. Sem retenção de dados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>OpenAI API</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>GPT-4o/mini</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>OpenAI ToS</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Output pertence ao cliente. Sem fine-tune lock.</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Comercial OK via API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Google Gemini API</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Flash/Pro</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Google AI ToS</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Free tier tem restrições. Paid tier = comercial OK.</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Verificar tier correto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Manus AI</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Pro Extended</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Manus ToS</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>SaaS</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Verificar cláusula de sublicenciamento.</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>64K tokens/mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Modelos Open-Weight (treinamento / on-prem)</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr"/>
+      <c r="C63" s="2" t="inlineStr"/>
+      <c r="D63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Qwen 3.5 27B</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>27B params</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Model weights</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Comercial sem restrições.</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Nosso SFT treinado em cima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Qwen 3 (se migrar)</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>vários</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0 / Qwen</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Model weights</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Qwen License = Apache-like. Comercial OK.</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Verificar versão específica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Llama 3.x (alternativa)</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>vários</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Meta Llama License</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Model weights</t>
+        </is>
+      </c>
+      <c r="E66" s="28" t="inlineStr">
+        <is>
+          <t>⚠ Condicional</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Grátis se &lt;700M MAU. Acima = licença Meta.</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Verificar threshold de usuários.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Mistral (alternativa)</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>vários</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Model weights</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Comercial sem restrições.</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Alternativa européia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>DeepSeek (alternativa)</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>R1/V3</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Model weights</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Comercial sem restrições.</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Alternativa chinesa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="27" t="inlineStr">
+        <is>
+          <t>🔧 TOOLING DE DESENVOLVIMENTO (não vai pro produto)</t>
+        </is>
+      </c>
+      <c r="B70" s="27" t="inlineStr"/>
+      <c r="C70" s="27" t="inlineStr"/>
+      <c r="D70" s="27" t="inlineStr"/>
+      <c r="E70" s="27" t="inlineStr"/>
+      <c r="F70" s="27" t="inlineStr"/>
+      <c r="G70" s="27" t="inlineStr"/>
+      <c r="H70" s="27" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas internas — usadas por nós, não entregues ao cliente</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr"/>
+      <c r="C71" s="2" t="inlineStr"/>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Agent framework</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Self-hosted, OSS.</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Nosso orchestrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>GitNexus</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Code intelligence</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Local only.</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Não vai pro deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Codex CLI (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>OpenAI ToS</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Dev tool</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>Pago por uso.</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>Code execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Cursor ToS</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>IDE</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Assinatura pessoal.</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Dev productivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Linear ToS</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>PM tool</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>$18/mês.</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Project management</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>GitHub ToS</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>VCS</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>Repo privado.</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Code hosting</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Jira/Confluence</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Atlassian Cloud ToS</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>PM/Docs</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>Free tier.</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="27" t="inlineStr">
+        <is>
+          <t>📋 RESUMO EXECUTIVO</t>
+        </is>
+      </c>
+      <c r="B81" s="27" t="inlineStr"/>
+      <c r="C81" s="27" t="inlineStr"/>
+      <c r="D81" s="27" t="inlineStr"/>
+      <c r="E81" s="27" t="inlineStr"/>
+      <c r="F81" s="27" t="inlineStr"/>
+      <c r="G81" s="27" t="inlineStr"/>
+      <c r="H81" s="27" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t>Total de dependências diretas</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>6 Python + 12 JS + 9 infra + 4 LLM APIs</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr"/>
+      <c r="E82" s="3" t="inlineStr"/>
+      <c r="F82" s="3" t="inlineStr"/>
+      <c r="G82" s="3" t="inlineStr"/>
+      <c r="H82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t>Total transitivas (npm)</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>112 pacotes</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr"/>
+      <c r="E83" s="3" t="inlineStr"/>
+      <c r="F83" s="3" t="inlineStr"/>
+      <c r="G83" s="3" t="inlineStr"/>
+      <c r="H83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>Licenças permissivas (MIT/BSD/Apache/ISC)</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>110 de 112 (98%)</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr"/>
+      <c r="D84" s="3" t="inlineStr"/>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr"/>
+      <c r="H84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>Licenças LGPL</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>2 de 112 (sharp/libvips)</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr"/>
+      <c r="D85" s="3" t="inlineStr"/>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Link dinâmico = OK comercial</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>Não modificamos o código</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>Licenças GPL / AGPL / SSPL</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112 (0%)</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr"/>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>NENHUMA</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Zero risco copyleft</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>Código proprietário nosso</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>100% do core (kernel, agentes, RAG, routing)</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr"/>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>Nosso IP total</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="inlineStr">
+        <is>
+          <t>Modelo SFT (Qwen 27B)</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Apache-2.0 base + nosso fine-tune</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr"/>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>Comercial sem restrição</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="19" t="inlineStr">
+        <is>
+          <t>✅ VEREDITO</t>
+        </is>
+      </c>
+      <c r="B90" s="19" t="inlineStr">
+        <is>
+          <t>APROVADO para comercialização. Zero licenças copyleft no runtime. 2 LGPL transitivas (sharp) são link dinâmico = permitido. LLM APIs pagas permitem uso comercial. Modelo Qwen é Apache-2.0.</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr"/>
+      <c r="D90" s="19" t="inlineStr"/>
+      <c r="E90" s="19" t="inlineStr"/>
+      <c r="F90" s="19" t="inlineStr"/>
+      <c r="G90" s="19" t="inlineStr"/>
+      <c r="H90" s="19" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="24" t="inlineStr">
+        <is>
+          <t>⚠ AÇÕES REQUERIDAS</t>
+        </is>
+      </c>
+      <c r="B92" s="24" t="inlineStr">
+        <is>
+          <t>1) Criar arquivo THIRD-PARTY-NOTICES com copyrights (MIT/BSD exigem). 2) Verificar ToS do Manus para sublicenciamento. 3) Se usar Llama: verificar threshold 700M MAU. 4) Se on-prem Mac Mini: incluir EULA para software Paganini.</t>
+        </is>
+      </c>
+      <c r="C92" s="24" t="inlineStr"/>
+      <c r="D92" s="24" t="inlineStr"/>
+      <c r="E92" s="24" t="inlineStr"/>
+      <c r="F92" s="24" t="inlineStr"/>
+      <c r="G92" s="24" t="inlineStr"/>
+      <c r="H92" s="24" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>